<commit_message>
Update apartment signature statuses
</commit_message>
<xml_diff>
--- a/governance/owner-signatures-2026.xlsx
+++ b/governance/owner-signatures-2026.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="90">
   <si>
     <t>חתימות בעלי דירות לבחירת ועד חדש</t>
   </si>
@@ -285,6 +285,9 @@
   </si>
   <si>
     <t>‎052-332-6597</t>
+  </si>
+  <si>
+    <t>2026-06-28</t>
   </si>
 </sst>
 </file>
@@ -585,7 +588,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <pageSetUpPr/>
   </sheetPr>
@@ -653,41 +656,41 @@
       </c>
     </row>
     <row r="4" ht="22.5" customHeight="1">
-      <c r="A4" s="4">
+      <c r="A4" s="6">
         <v>1.0</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="K4" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="L4" s="4" t="s">
-        <v>17</v>
+      <c r="E4" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="L4" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="5" ht="22.5" customHeight="1">
@@ -729,41 +732,41 @@
       </c>
     </row>
     <row r="6" ht="22.5" customHeight="1">
-      <c r="A6" s="4">
+      <c r="A6" s="6">
         <v>3.0</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="J6" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="K6" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="L6" s="4" t="s">
-        <v>17</v>
+      <c r="E6" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="J6" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="L6" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="7" ht="22.5" customHeight="1">
@@ -881,41 +884,41 @@
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1">
-      <c r="A10" s="4">
+      <c r="A10" s="6">
         <v>7.0</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="E10" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="H10" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="K10" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="L10" s="4" t="s">
-        <v>17</v>
+      <c r="E10" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="I10" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="J10" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="K10" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="L10" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="11" ht="22.5" customHeight="1">
@@ -2482,6 +2485,6 @@
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
+  <drawing ns1:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Mark apartment 5 signed
</commit_message>
<xml_diff>
--- a/governance/owner-signatures-2026.xlsx
+++ b/governance/owner-signatures-2026.xlsx
@@ -808,41 +808,41 @@
       </c>
     </row>
     <row r="8" ht="22.5" customHeight="1">
-      <c r="A8" s="4">
+      <c r="A8" s="6">
         <v>5.0</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="J8" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="K8" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="L8" s="4" t="s">
-        <v>17</v>
+      <c r="E8" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="J8" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="K8" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="L8" s="7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="9" ht="22.5" customHeight="1">

</xml_diff>

<commit_message>
Add apartment 6 signature document
</commit_message>
<xml_diff>
--- a/governance/owner-signatures-2026.xlsx
+++ b/governance/owner-signatures-2026.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="93">
   <si>
     <t>חתימות בעלי דירות לבחירת ועד חדש</t>
   </si>
@@ -288,6 +288,15 @@
   </si>
   <si>
     <t>2026-06-28</t>
+  </si>
+  <si>
+    <t>2026-06-30</t>
+  </si>
+  <si>
+    <t>מסמך Telegram</t>
+  </si>
+  <si>
+    <t>documents/apartment-6-signature-2026-06-30.pdf</t>
   </si>
 </sst>
 </file>
@@ -846,40 +855,40 @@
       </c>
     </row>
     <row r="9" ht="22.5" customHeight="1">
-      <c r="A9" s="4">
+      <c r="A9" s="6">
         <v>6.0</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="E9" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="J9" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="K9" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="L9" s="4" t="s">
+      <c r="E9" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="J9" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="L9" s="6" t="s">
         <v>17</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add apartment 18 signature document
</commit_message>
<xml_diff>
--- a/governance/owner-signatures-2026.xlsx
+++ b/governance/owner-signatures-2026.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="94">
   <si>
     <t>חתימות בעלי דירות לבחירת ועד חדש</t>
   </si>
@@ -297,6 +297,9 @@
   </si>
   <si>
     <t>documents/apartment-6-signature-2026-06-30.pdf</t>
+  </si>
+  <si>
+    <t>documents/apartment-18-signature-2026-06-30.pdf</t>
   </si>
 </sst>
 </file>
@@ -1395,40 +1398,40 @@
       <c r="Z20" s="6"/>
     </row>
     <row r="21" ht="22.5" customHeight="1">
-      <c r="A21" s="4">
+      <c r="A21" s="6">
         <v>18.0</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="C21" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D21" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="E21" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="F21" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="G21" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="H21" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="I21" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="J21" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="K21" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="L21" s="4" t="s">
+      <c r="E21" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H21" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="I21" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="J21" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="K21" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="L21" s="6" t="s">
         <v>17</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Mark apartments 11 and 19 signed
</commit_message>
<xml_diff>
--- a/governance/owner-signatures-2026.xlsx
+++ b/governance/owner-signatures-2026.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="95">
   <si>
     <t>חתימות בעלי דירות לבחירת ועד חדש</t>
   </si>
@@ -300,6 +300,9 @@
   </si>
   <si>
     <t>documents/apartment-18-signature-2026-06-30.pdf</t>
+  </si>
+  <si>
+    <t>2026-07-03</t>
   </si>
 </sst>
 </file>
@@ -1062,41 +1065,41 @@
       <c r="Z13" s="6"/>
     </row>
     <row r="14" ht="22.5" customHeight="1">
-      <c r="A14" s="4">
+      <c r="A14" s="6">
         <v>11.0</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="E14" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="H14" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="I14" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="J14" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="K14" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="L14" s="4" t="s">
-        <v>17</v>
+      <c r="E14" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H14" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="I14" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="J14" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="K14" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="L14" s="6" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="15" ht="22.5" customHeight="1">
@@ -1436,41 +1439,41 @@
       </c>
     </row>
     <row r="22" ht="22.5" customHeight="1">
-      <c r="A22" s="4">
+      <c r="A22" s="6">
         <v>19.0</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="B22" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="C22" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="D22" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="E22" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="G22" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="H22" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="I22" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="J22" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="K22" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="L22" s="4" t="s">
-        <v>17</v>
+      <c r="E22" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H22" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="I22" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="J22" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="K22" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="L22" s="6" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="23" ht="22.5" customHeight="1">

</xml_diff>

<commit_message>
Mark apartment 9 signed
</commit_message>
<xml_diff>
--- a/governance/owner-signatures-2026.xlsx
+++ b/governance/owner-signatures-2026.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="102">
   <si>
     <t>חתימות בעלי דירות לבחירת ועד חדש</t>
   </si>
@@ -312,6 +312,18 @@
   </si>
   <si>
     <t>מסמך חתום התקבל ב-Telegram; דירה 8</t>
+  </si>
+  <si>
+    <t>עודכן: 2026-07-07</t>
+  </si>
+  <si>
+    <t>ועד בית</t>
+  </si>
+  <si>
+    <t>2026-07-07</t>
+  </si>
+  <si>
+    <t>אושר בהודעת Telegram ללא קובץ מצורף; דירה 15 היא ועד בית</t>
   </si>
 </sst>
 </file>
@@ -612,7 +624,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <pageSetUpPr/>
   </sheetPr>
@@ -637,8 +649,10 @@
       </c>
     </row>
     <row r="2" ht="22.5" customHeight="1">
-      <c r="A2" s="2" t="s">
-        <v>1</v>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>עודכן: 2026-07-08</t>
+        </is>
       </c>
     </row>
     <row r="3" ht="24.75" customHeight="1">
@@ -1005,20 +1019,30 @@
       <c r="G12" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="H12" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="I12" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="J12" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="K12" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="L12" s="4" t="s">
-        <v>17</v>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>נחתם</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>מסמך Telegram</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>documents/apartment-9-signature-2026-07-08.pdf</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t>מסמך חתום התקבל ב-Telegram; דירה 9</t>
+        </is>
       </c>
     </row>
     <row r="13" ht="22.5" customHeight="1">
@@ -1268,41 +1292,41 @@
       <c r="Z17" s="6"/>
     </row>
     <row r="18" ht="22.5" customHeight="1">
-      <c r="A18" s="4">
+      <c r="A18" s="6">
         <v>15.0</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="C18" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="D18" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="E18" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="F18" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="G18" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="H18" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="I18" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="J18" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="K18" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="L18" s="4" t="s">
-        <v>17</v>
+      <c r="E18" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="I18" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="J18" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="K18" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="L18" s="6" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="19" ht="22.5" customHeight="1">
@@ -2509,6 +2533,6 @@
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing ns1:id="rId1"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>